<commit_message>
INPUT_V8.xlsx: remove extra spaces inside five teacher names
Rows 7, 8, 23, 35 and 36 of NHÂN SỰ had two spaces between words of the
name. Only those five shared strings were edited in the xlsx XML; every
other cell, style and sheet is unchanged, and the staff list (titles,
roles, classes, lessons) and curriculum read exactly as before, so the
timetable and result codes do not change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/INPUT_V8.xlsx
+++ b/data/INPUT_V8.xlsx
@@ -315,19 +315,19 @@
     <t>3/5</t>
   </si>
   <si>
-    <t>Nguyễn Thị Xuân  Lộc</t>
-  </si>
-  <si>
-    <t>Lê Thị  Lạc</t>
-  </si>
-  <si>
-    <t>Nguyễn Văn  Nuôi</t>
-  </si>
-  <si>
-    <t>Nguyễn Ngọc Phương  Quỳnh</t>
-  </si>
-  <si>
-    <t>Trương Thị  Hạnh</t>
+    <t>Nguyễn Thị Xuân Lộc</t>
+  </si>
+  <si>
+    <t>Lê Thị Lạc</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn Nuôi</t>
+  </si>
+  <si>
+    <t>Nguyễn Ngọc Phương Quỳnh</t>
+  </si>
+  <si>
+    <t>Trương Thị Hạnh</t>
   </si>
   <si>
     <t>Nguyễn Thị Phụng</t>

</xml_diff>

<commit_message>
Drop the duplicated staff row; overtime up to 3 in main.py
Row 34 of the school file (general teacher, 23 lessons) is the same
person as row 46 (general teacher on maternity leave); the school
confirmed it and the row is removed (44 staff). Without those 23
lessons, overtime capped at 2 leaves 17 lessons uncovered (music 6,
art 6, technology 4, life skills 1), so the school set
SO_TIET_BU_TOI_DA to 3: the estimate is 79 overtime lessons, all by
homeroom teachers (23 at +3, 5 at +2). config.OVERTIME_MAX (CLI and
tests) stays 2; the sample school's assignment is identical at +3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/INPUT_V8.xlsx
+++ b/data/INPUT_V8.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18.75"/>
   <cols>
     <col width="33.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1428,12 +1428,12 @@
     <row r="34" ht="24.95" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Trúc Ly</t>
+          <t>Nguyễn Ngọc Phương Quỳnh</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Bộ Môn</t>
+          <t xml:space="preserve">Tiếng Anh </t>
         </is>
       </c>
       <c r="C34" s="9" t="n"/>
@@ -1443,77 +1443,89 @@
       <c r="E34" s="13" t="n"/>
       <c r="F34" s="14" t="n"/>
       <c r="G34" s="15" t="n"/>
-      <c r="H34" s="17" t="n"/>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>3D18, 3D19, 3D20, 3D21, 3D22, 3D23</t>
+        </is>
+      </c>
       <c r="I34" s="15" t="n"/>
     </row>
     <row r="35" ht="24.95" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Phương Quỳnh</t>
+          <t>Trương Thị Hạnh</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiếng Anh </t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="n"/>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>5D22</t>
+        </is>
+      </c>
       <c r="D35" s="13" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E35" s="13" t="n"/>
       <c r="F35" s="14" t="n"/>
-      <c r="G35" s="15" t="n"/>
-      <c r="H35" s="17" t="inlineStr">
-        <is>
-          <t>3D18, 3D19, 3D20, 3D21, 3D22, 3D23</t>
-        </is>
-      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="H35" s="17" t="n"/>
       <c r="I35" s="15" t="n"/>
     </row>
     <row r="36" ht="24.95" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Trương Thị Hạnh</t>
+          <t>Nguyễn Thị Ái Phi</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>5D22</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Tiếng Anh </t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="n"/>
       <c r="D36" s="13" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E36" s="13" t="n"/>
-      <c r="F36" s="14" t="n"/>
-      <c r="G36" s="15" t="inlineStr">
+      <c r="F36" s="15" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="H36" s="17" t="n"/>
+      <c r="G36" s="15" t="n"/>
+      <c r="H36" s="17" t="inlineStr">
+        <is>
+          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D18, 2D19, 2D20, 2D21, 3D19, 3D20, 3D21, 3D22, 3D23</t>
+        </is>
+      </c>
       <c r="I36" s="15" t="n"/>
     </row>
     <row r="37" ht="24.95" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Ái Phi</t>
+          <t>Lê Thị Hạnh Nhân</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiếng Anh </t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="n"/>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>4D22</t>
+        </is>
+      </c>
       <c r="D37" s="13" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E37" s="13" t="n"/>
       <c r="F37" s="15" t="inlineStr">
@@ -1521,32 +1533,28 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G37" s="15" t="n"/>
-      <c r="H37" s="17" t="inlineStr">
-        <is>
-          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D18, 2D19, 2D20, 2D21, 3D19, 3D20, 3D21, 3D22, 3D23</t>
-        </is>
-      </c>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="H37" s="17" t="n"/>
       <c r="I37" s="15" t="n"/>
     </row>
     <row r="38" ht="24.95" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Lê Thị Hạnh Nhân</t>
+          <t>Võ Thị Luyến</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>4D22</t>
-        </is>
-      </c>
+          <t>Bộ Môn</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="n"/>
       <c r="D38" s="13" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E38" s="13" t="n"/>
       <c r="F38" s="15" t="inlineStr">
@@ -1554,18 +1562,18 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G38" s="15" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="H38" s="17" t="n"/>
+      <c r="G38" s="15" t="n"/>
+      <c r="H38" s="17" t="inlineStr">
+        <is>
+          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 5D18</t>
+        </is>
+      </c>
       <c r="I38" s="15" t="n"/>
     </row>
     <row r="39" ht="24.95" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Võ Thị Luyến</t>
+          <t>Lê Thị Bửu Châu</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -1586,7 +1594,7 @@
       <c r="G39" s="15" t="n"/>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 5D18</t>
+          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 3D17, 3D18, 3D23</t>
         </is>
       </c>
       <c r="I39" s="15" t="n"/>
@@ -1594,17 +1602,21 @@
     <row r="40" ht="24.95" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Lê Thị Bửu Châu</t>
+          <t>Nguyễn Thị Tý</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Bộ Môn</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="n"/>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>2D20</t>
+        </is>
+      </c>
       <c r="D40" s="13" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E40" s="13" t="n"/>
       <c r="F40" s="15" t="inlineStr">
@@ -1613,31 +1625,23 @@
         </is>
       </c>
       <c r="G40" s="15" t="n"/>
-      <c r="H40" s="17" t="inlineStr">
-        <is>
-          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 3D17, 3D18, 3D23</t>
-        </is>
-      </c>
+      <c r="H40" s="17" t="n"/>
       <c r="I40" s="15" t="n"/>
     </row>
     <row r="41" ht="24.95" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Tý</t>
+          <t>Nguyễn Thuận An</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C41" s="10" t="inlineStr">
-        <is>
-          <t>2D20</t>
-        </is>
-      </c>
+          <t>Bộ Môn</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="n"/>
       <c r="D41" s="13" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E41" s="13" t="n"/>
       <c r="F41" s="15" t="inlineStr">
@@ -1646,23 +1650,31 @@
         </is>
       </c>
       <c r="G41" s="15" t="n"/>
-      <c r="H41" s="17" t="n"/>
+      <c r="H41" s="17" t="inlineStr">
+        <is>
+          <t>2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D22, 5D18</t>
+        </is>
+      </c>
       <c r="I41" s="15" t="n"/>
     </row>
     <row r="42" ht="24.95" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thuận An</t>
+          <t>Phạm Hồ Hải Oanh</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Bộ Môn</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="n"/>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>3D22</t>
+        </is>
+      </c>
       <c r="D42" s="13" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E42" s="13" t="n"/>
       <c r="F42" s="15" t="inlineStr">
@@ -1670,32 +1682,28 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G42" s="15" t="n"/>
-      <c r="H42" s="17" t="inlineStr">
-        <is>
-          <t>2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D22, 5D18</t>
-        </is>
-      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="H42" s="17" t="n"/>
       <c r="I42" s="15" t="n"/>
     </row>
     <row r="43" ht="24.95" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Phạm Hồ Hải Oanh</t>
+          <t>Lưu Thành Vũ</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>3D22</t>
-        </is>
-      </c>
+          <t>Tin học</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="n"/>
       <c r="D43" s="13" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E43" s="13" t="n"/>
       <c r="F43" s="15" t="inlineStr">
@@ -1703,23 +1711,23 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G43" s="15" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="H43" s="17" t="n"/>
+      <c r="G43" s="15" t="n"/>
+      <c r="H43" s="17" t="inlineStr">
+        <is>
+          <t>3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D18, 4D19, 4D20, 4D21, 4D22, 5D18, 5D19, 5D20, 5D21, 5D22</t>
+        </is>
+      </c>
       <c r="I43" s="15" t="n"/>
     </row>
     <row r="44" ht="24.95" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Lưu Thành Vũ</t>
+          <t>Lê Hoàng Khoa</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Tin học</t>
+          <t>Thể dục</t>
         </is>
       </c>
       <c r="C44" s="9" t="n"/>
@@ -1735,7 +1743,7 @@
       <c r="G44" s="15" t="n"/>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D18, 4D19, 4D20, 4D21, 4D22, 5D18, 5D19, 5D20, 5D21, 5D22</t>
+          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 5D18, 5D19, 5D20, 5D21, 5D22</t>
         </is>
       </c>
       <c r="I44" s="15" t="n"/>
@@ -1743,61 +1751,33 @@
     <row r="45" ht="24.95" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Lê Hoàng Khoa</t>
+          <t>Nguyễn Thị Trúc Ly</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Thể dục</t>
+          <t>Bộ Môn</t>
         </is>
       </c>
       <c r="C45" s="9" t="n"/>
       <c r="D45" s="13" t="n">
-        <v>23</v>
-      </c>
-      <c r="E45" s="13" t="n"/>
-      <c r="F45" s="15" t="inlineStr">
+        <v>19</v>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
+      <c r="F45" s="14" t="n"/>
       <c r="G45" s="15" t="n"/>
-      <c r="H45" s="17" t="inlineStr">
-        <is>
-          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 5D18, 5D19, 5D20, 5D21, 5D22</t>
-        </is>
-      </c>
-      <c r="I45" s="15" t="n"/>
-    </row>
-    <row r="46" ht="24.95" customHeight="1">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>Nguyễn Thị Trúc Ly</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Bộ Môn</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="n"/>
-      <c r="D46" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="E46" s="13" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="F46" s="14" t="n"/>
-      <c r="G46" s="15" t="n"/>
-      <c r="H46" s="17" t="n"/>
-      <c r="I46" s="15" t="inlineStr">
+      <c r="H45" s="17" t="n"/>
+      <c r="I45" s="15" t="inlineStr">
         <is>
           <t>Chiều T5, Sáng T6</t>
         </is>
       </c>
     </row>
+    <row r="46" ht="24.95" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
New school file: duplicate merged into row 34
The school sent a corrected input: the duplicated general teacher is now
one row (row 34, the maternity teacher with 19 lessons, campus 2), row 46
is gone, 44 staff. Its file has no Lớp Đang Dạy / Buổi Nghỉ columns, so
both are copied over from the previous file, matched by name (14 rows of
old classes; leave for the homeroom teacher of 3D23 and for row 34).
The estimate is unchanged (79 overtime lessons); result codes change
with the row order and are updated once the runs finish.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/INPUT_V8.xlsx
+++ b/data/INPUT_V8.xlsx
@@ -77,7 +77,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -126,11 +126,61 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF505050"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF505050"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF505050"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF505050"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF505050"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF505050"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -174,6 +224,40 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -544,21 +628,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="18.75"/>
+  <dimension ref="A1:I46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col width="33.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="7" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="16.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="11.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="10.42578125" bestFit="1" customWidth="1" style="16" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="33.62890625" bestFit="1" customWidth="1" style="20" min="1" max="1"/>
+    <col width="13.44921875" bestFit="1" customWidth="1" style="20" min="2" max="2"/>
+    <col width="6.9921875" bestFit="1" customWidth="1" style="20" min="3" max="3"/>
+    <col width="16.6796875" bestFit="1" customWidth="1" style="20" min="4" max="4"/>
+    <col width="11.8359375" bestFit="1" customWidth="1" style="20" min="5" max="5"/>
+    <col width="13.44921875" bestFit="1" customWidth="1" style="20" min="6" max="6"/>
+    <col width="10.35546875" bestFit="1" customWidth="1" style="19" min="7" max="7"/>
+    <col width="40" customWidth="1" style="20" min="8" max="8"/>
+    <col width="22" customWidth="1" style="20" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24.95" customHeight="1">
+    <row r="1" ht="24.95" customHeight="1" s="20">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Họ và Tên</t>
@@ -605,7 +689,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="24.95" customHeight="1">
+    <row r="2" ht="24.95" customHeight="1" s="20">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Thân Tấn Tâm</t>
@@ -623,14 +707,14 @@
       <c r="E2" s="13" t="n"/>
       <c r="F2" s="14" t="n"/>
       <c r="G2" s="15" t="n"/>
-      <c r="H2" s="17" t="inlineStr">
+      <c r="H2" s="29" t="inlineStr">
         <is>
           <t>4D18, 4D19, 4D20</t>
         </is>
       </c>
       <c r="I2" s="15" t="n"/>
     </row>
-    <row r="3" ht="24.95" customHeight="1">
+    <row r="3" ht="24.95" customHeight="1" s="20">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Võ Thị Thu Ngọc</t>
@@ -652,10 +736,10 @@
       <c r="E3" s="13" t="n"/>
       <c r="F3" s="14" t="n"/>
       <c r="G3" s="15" t="n"/>
-      <c r="H3" s="17" t="n"/>
+      <c r="H3" s="29" t="n"/>
       <c r="I3" s="15" t="n"/>
     </row>
-    <row r="4" ht="24.95" customHeight="1">
+    <row r="4" ht="24.95" customHeight="1" s="20">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Trần Thùy Dương</t>
@@ -677,10 +761,10 @@
       <c r="E4" s="13" t="n"/>
       <c r="F4" s="14" t="n"/>
       <c r="G4" s="15" t="n"/>
-      <c r="H4" s="17" t="n"/>
+      <c r="H4" s="29" t="n"/>
       <c r="I4" s="15" t="n"/>
     </row>
-    <row r="5" ht="24.95" customHeight="1">
+    <row r="5" ht="24.95" customHeight="1" s="20">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Đoàn Tuấn Anh</t>
@@ -698,14 +782,14 @@
       <c r="E5" s="13" t="n"/>
       <c r="F5" s="14" t="n"/>
       <c r="G5" s="15" t="n"/>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="H5" s="29" t="inlineStr">
         <is>
           <t>1D16, 1D17, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 4D18, 4D19, 4D20, 4D21, 4D22</t>
         </is>
       </c>
       <c r="I5" s="15" t="n"/>
     </row>
-    <row r="6" ht="24.95" customHeight="1">
+    <row r="6" ht="24.95" customHeight="1" s="20">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Ngô Thị Hoàng Viễn</t>
@@ -727,10 +811,10 @@
       <c r="E6" s="13" t="n"/>
       <c r="F6" s="14" t="n"/>
       <c r="G6" s="15" t="n"/>
-      <c r="H6" s="17" t="n"/>
+      <c r="H6" s="29" t="n"/>
       <c r="I6" s="15" t="n"/>
     </row>
-    <row r="7" ht="24.95" customHeight="1">
+    <row r="7" ht="24.95" customHeight="1" s="20">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Thị Xuân Lộc</t>
@@ -752,10 +836,10 @@
       <c r="E7" s="13" t="n"/>
       <c r="F7" s="14" t="n"/>
       <c r="G7" s="15" t="n"/>
-      <c r="H7" s="17" t="n"/>
+      <c r="H7" s="29" t="n"/>
       <c r="I7" s="15" t="n"/>
     </row>
-    <row r="8" ht="24.95" customHeight="1">
+    <row r="8" ht="24.95" customHeight="1" s="20">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Lê Thị Lạc</t>
@@ -777,10 +861,10 @@
       <c r="E8" s="13" t="n"/>
       <c r="F8" s="14" t="n"/>
       <c r="G8" s="15" t="n"/>
-      <c r="H8" s="17" t="n"/>
+      <c r="H8" s="29" t="n"/>
       <c r="I8" s="15" t="n"/>
     </row>
-    <row r="9" ht="24.95" customHeight="1">
+    <row r="9" ht="24.95" customHeight="1" s="20">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Thị Phụng</t>
@@ -802,10 +886,10 @@
       <c r="E9" s="13" t="n"/>
       <c r="F9" s="14" t="n"/>
       <c r="G9" s="15" t="n"/>
-      <c r="H9" s="17" t="n"/>
+      <c r="H9" s="29" t="n"/>
       <c r="I9" s="15" t="n"/>
     </row>
-    <row r="10" ht="24.95" customHeight="1">
+    <row r="10" ht="24.95" customHeight="1" s="20">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Lê Nguyễn Bảo Hòa</t>
@@ -823,14 +907,14 @@
       <c r="E10" s="13" t="n"/>
       <c r="F10" s="14" t="n"/>
       <c r="G10" s="15" t="n"/>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="H10" s="29" t="inlineStr">
         <is>
           <t>3D17, 4D18, 4D19, 4D20, 4D21, 4D22</t>
         </is>
       </c>
       <c r="I10" s="15" t="n"/>
     </row>
-    <row r="11" ht="24.95" customHeight="1">
+    <row r="11" ht="24.95" customHeight="1" s="20">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Đỗ Thị Dung</t>
@@ -852,10 +936,10 @@
       <c r="E11" s="13" t="n"/>
       <c r="F11" s="14" t="n"/>
       <c r="G11" s="15" t="n"/>
-      <c r="H11" s="17" t="n"/>
+      <c r="H11" s="29" t="n"/>
       <c r="I11" s="15" t="n"/>
     </row>
-    <row r="12" ht="24.95" customHeight="1">
+    <row r="12" ht="24.95" customHeight="1" s="20">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Võ Thị Tú Vân</t>
@@ -881,10 +965,10 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="H12" s="17" t="n"/>
+      <c r="H12" s="29" t="n"/>
       <c r="I12" s="15" t="n"/>
     </row>
-    <row r="13" ht="24.95" customHeight="1">
+    <row r="13" ht="24.95" customHeight="1" s="20">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Lê Thụy Linh Sa</t>
@@ -902,14 +986,14 @@
       <c r="E13" s="13" t="n"/>
       <c r="F13" s="14" t="n"/>
       <c r="G13" s="15" t="n"/>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="H13" s="29" t="inlineStr">
         <is>
           <t>2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D18, 4D19, 4D20, 4D21, 4D22, 5D18, 5D19, 5D20, 5D21, 5D22</t>
         </is>
       </c>
       <c r="I13" s="15" t="n"/>
     </row>
-    <row r="14" ht="24.95" customHeight="1">
+    <row r="14" ht="24.95" customHeight="1" s="20">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Huỳnh Thị Tường Vi</t>
@@ -931,10 +1015,10 @@
       <c r="E14" s="13" t="n"/>
       <c r="F14" s="14" t="n"/>
       <c r="G14" s="15" t="n"/>
-      <c r="H14" s="17" t="n"/>
+      <c r="H14" s="29" t="n"/>
       <c r="I14" s="15" t="n"/>
     </row>
-    <row r="15" ht="24.95" customHeight="1">
+    <row r="15" ht="24.95" customHeight="1" s="20">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Thị Kiều Oanh</t>
@@ -956,10 +1040,10 @@
       <c r="E15" s="13" t="n"/>
       <c r="F15" s="14" t="n"/>
       <c r="G15" s="15" t="n"/>
-      <c r="H15" s="17" t="n"/>
+      <c r="H15" s="29" t="n"/>
       <c r="I15" s="15" t="n"/>
     </row>
-    <row r="16" ht="24.95" customHeight="1">
+    <row r="16" ht="24.95" customHeight="1" s="20">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Đoàn Thịnh</t>
@@ -977,14 +1061,14 @@
       <c r="E16" s="13" t="n"/>
       <c r="F16" s="14" t="n"/>
       <c r="G16" s="15" t="n"/>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="H16" s="29" t="inlineStr">
         <is>
           <t>1D15, 3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 5D18, 5D19, 5D20, 5D21, 5D22</t>
         </is>
       </c>
       <c r="I16" s="15" t="n"/>
     </row>
-    <row r="17" ht="24.95" customHeight="1">
+    <row r="17" ht="24.95" customHeight="1" s="20">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Trần Thị Kim Ngọc</t>
@@ -1010,10 +1094,10 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="H17" s="17" t="n"/>
+      <c r="H17" s="29" t="n"/>
       <c r="I17" s="15" t="n"/>
     </row>
-    <row r="18" ht="24.95" customHeight="1">
+    <row r="18" ht="24.95" customHeight="1" s="20">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Thị Thu Trang</t>
@@ -1035,10 +1119,10 @@
       <c r="E18" s="13" t="n"/>
       <c r="F18" s="14" t="n"/>
       <c r="G18" s="15" t="n"/>
-      <c r="H18" s="17" t="n"/>
+      <c r="H18" s="29" t="n"/>
       <c r="I18" s="15" t="n"/>
     </row>
-    <row r="19" ht="24.95" customHeight="1">
+    <row r="19" ht="24.95" customHeight="1" s="20">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Phạm Thị Hồng Nhung</t>
@@ -1060,10 +1144,10 @@
       <c r="E19" s="13" t="n"/>
       <c r="F19" s="14" t="n"/>
       <c r="G19" s="15" t="n"/>
-      <c r="H19" s="17" t="n"/>
+      <c r="H19" s="29" t="n"/>
       <c r="I19" s="15" t="n"/>
     </row>
-    <row r="20" ht="24.95" customHeight="1">
+    <row r="20" ht="24.95" customHeight="1" s="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Trần Thị Giang Thảo</t>
@@ -1085,10 +1169,10 @@
       <c r="E20" s="13" t="n"/>
       <c r="F20" s="14" t="n"/>
       <c r="G20" s="15" t="n"/>
-      <c r="H20" s="17" t="n"/>
+      <c r="H20" s="29" t="n"/>
       <c r="I20" s="15" t="n"/>
     </row>
-    <row r="21" ht="24.95" customHeight="1">
+    <row r="21" ht="24.95" customHeight="1" s="20">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Trương Minh Trân</t>
@@ -1110,10 +1194,10 @@
       <c r="E21" s="13" t="n"/>
       <c r="F21" s="14" t="n"/>
       <c r="G21" s="15" t="n"/>
-      <c r="H21" s="17" t="n"/>
+      <c r="H21" s="29" t="n"/>
       <c r="I21" s="15" t="n"/>
     </row>
-    <row r="22" ht="24.95" customHeight="1">
+    <row r="22" ht="24.95" customHeight="1" s="20">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Thị Phước Tri</t>
@@ -1135,10 +1219,10 @@
       <c r="E22" s="13" t="n"/>
       <c r="F22" s="14" t="n"/>
       <c r="G22" s="15" t="n"/>
-      <c r="H22" s="17" t="n"/>
+      <c r="H22" s="29" t="n"/>
       <c r="I22" s="15" t="n"/>
     </row>
-    <row r="23" ht="24.95" customHeight="1">
+    <row r="23" ht="24.95" customHeight="1" s="20">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Văn Nuôi</t>
@@ -1160,10 +1244,10 @@
       <c r="E23" s="13" t="n"/>
       <c r="F23" s="14" t="n"/>
       <c r="G23" s="15" t="n"/>
-      <c r="H23" s="17" t="n"/>
+      <c r="H23" s="29" t="n"/>
       <c r="I23" s="15" t="n"/>
     </row>
-    <row r="24" ht="24.95" customHeight="1">
+    <row r="24" ht="24.95" customHeight="1" s="20">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Đặng Thị Ngọc Mai</t>
@@ -1193,14 +1277,14 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="H24" s="17" t="n"/>
+      <c r="H24" s="29" t="n"/>
       <c r="I24" s="15" t="inlineStr">
         <is>
           <t>2 buổi chiều</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24.95" customHeight="1">
+    <row r="25" ht="24.95" customHeight="1" s="20">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Bùi Thị Tường Vi</t>
@@ -1218,14 +1302,14 @@
       <c r="E25" s="13" t="n"/>
       <c r="F25" s="14" t="n"/>
       <c r="G25" s="15" t="n"/>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="H25" s="29" t="inlineStr">
         <is>
           <t>2D16, 2D17, 5D18, 5D19, 5D20, 5D21, 5D22</t>
         </is>
       </c>
       <c r="I25" s="15" t="n"/>
     </row>
-    <row r="26" ht="24.95" customHeight="1">
+    <row r="26" ht="24.95" customHeight="1" s="20">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Bùi Thị Thu Huyền</t>
@@ -1247,10 +1331,10 @@
       <c r="E26" s="13" t="n"/>
       <c r="F26" s="14" t="n"/>
       <c r="G26" s="15" t="n"/>
-      <c r="H26" s="17" t="n"/>
+      <c r="H26" s="29" t="n"/>
       <c r="I26" s="15" t="n"/>
     </row>
-    <row r="27" ht="24.95" customHeight="1">
+    <row r="27" ht="24.95" customHeight="1" s="20">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Trần Anh Thư</t>
@@ -1272,10 +1356,10 @@
       <c r="E27" s="13" t="n"/>
       <c r="F27" s="14" t="n"/>
       <c r="G27" s="15" t="n"/>
-      <c r="H27" s="17" t="n"/>
+      <c r="H27" s="29" t="n"/>
       <c r="I27" s="15" t="n"/>
     </row>
-    <row r="28" ht="24.95" customHeight="1">
+    <row r="28" ht="24.95" customHeight="1" s="20">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Trần Thị Thanh Huyền</t>
@@ -1297,10 +1381,10 @@
       <c r="E28" s="13" t="n"/>
       <c r="F28" s="14" t="n"/>
       <c r="G28" s="15" t="n"/>
-      <c r="H28" s="17" t="n"/>
+      <c r="H28" s="29" t="n"/>
       <c r="I28" s="15" t="n"/>
     </row>
-    <row r="29" ht="24.95" customHeight="1">
+    <row r="29" ht="24.95" customHeight="1" s="20">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Huỳnh Thị Kim Thu</t>
@@ -1318,14 +1402,14 @@
       <c r="E29" s="13" t="n"/>
       <c r="F29" s="14" t="n"/>
       <c r="G29" s="15" t="n"/>
-      <c r="H29" s="17" t="inlineStr">
+      <c r="H29" s="29" t="inlineStr">
         <is>
           <t>1D15, 1D16, 1D17, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D18, 4D19, 4D20, 4D21, 4D22, 5D18, 5D19, 5D20, 5D21, 5D22</t>
         </is>
       </c>
       <c r="I29" s="15" t="n"/>
     </row>
-    <row r="30" ht="24.95" customHeight="1">
+    <row r="30" ht="24.95" customHeight="1" s="20">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Thế Dân</t>
@@ -1347,10 +1431,10 @@
       <c r="E30" s="13" t="n"/>
       <c r="F30" s="14" t="n"/>
       <c r="G30" s="15" t="n"/>
-      <c r="H30" s="17" t="n"/>
+      <c r="H30" s="29" t="n"/>
       <c r="I30" s="15" t="n"/>
     </row>
-    <row r="31" ht="24.95" customHeight="1">
+    <row r="31" ht="24.95" customHeight="1" s="20">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Võ Thị Trúc Ly</t>
@@ -1372,10 +1456,10 @@
       <c r="E31" s="13" t="n"/>
       <c r="F31" s="14" t="n"/>
       <c r="G31" s="15" t="n"/>
-      <c r="H31" s="17" t="n"/>
+      <c r="H31" s="29" t="n"/>
       <c r="I31" s="15" t="n"/>
     </row>
-    <row r="32" ht="24.95" customHeight="1">
+    <row r="32" ht="24.95" customHeight="1" s="20">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Hoàng Vy</t>
@@ -1397,10 +1481,10 @@
       <c r="E32" s="13" t="n"/>
       <c r="F32" s="14" t="n"/>
       <c r="G32" s="15" t="n"/>
-      <c r="H32" s="17" t="n"/>
+      <c r="H32" s="29" t="n"/>
       <c r="I32" s="15" t="n"/>
     </row>
-    <row r="33" ht="24.95" customHeight="1">
+    <row r="33" ht="24.95" customHeight="1" s="20">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Lâm Thị Bích Thủy</t>
@@ -1422,110 +1506,110 @@
       <c r="E33" s="13" t="n"/>
       <c r="F33" s="14" t="n"/>
       <c r="G33" s="15" t="n"/>
-      <c r="H33" s="17" t="n"/>
+      <c r="H33" s="29" t="n"/>
       <c r="I33" s="15" t="n"/>
     </row>
-    <row r="34" ht="24.95" customHeight="1">
+    <row r="34" ht="24.95" customHeight="1" s="20">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Phương Quỳnh</t>
+          <t>Nguyễn Thị Trúc Ly</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiếng Anh </t>
+          <t>Bộ Môn</t>
         </is>
       </c>
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="n"/>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="H34" s="29" t="n"/>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>Chiều T5, Sáng T6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24.95" customHeight="1" s="20">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Nguyễn Ngọc Phương Quỳnh</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiếng Anh </t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="13" t="n">
         <v>23</v>
-      </c>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="15" t="n"/>
-      <c r="H34" s="17" t="inlineStr">
-        <is>
-          <t>3D18, 3D19, 3D20, 3D21, 3D22, 3D23</t>
-        </is>
-      </c>
-      <c r="I34" s="15" t="n"/>
-    </row>
-    <row r="35" ht="24.95" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>Trương Thị Hạnh</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>5D22</t>
-        </is>
-      </c>
-      <c r="D35" s="13" t="n">
-        <v>19</v>
       </c>
       <c r="E35" s="13" t="n"/>
       <c r="F35" s="14" t="n"/>
-      <c r="G35" s="15" t="inlineStr">
+      <c r="G35" s="15" t="n"/>
+      <c r="H35" s="29" t="inlineStr">
+        <is>
+          <t>3D18, 3D19, 3D20, 3D21, 3D22, 3D23</t>
+        </is>
+      </c>
+      <c r="I35" s="15" t="n"/>
+    </row>
+    <row r="36" ht="24.95" customHeight="1" s="20">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Trương Thị Hạnh</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>5D22</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="14" t="n"/>
+      <c r="G36" s="15" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="H35" s="17" t="n"/>
-      <c r="I35" s="15" t="n"/>
-    </row>
-    <row r="36" ht="24.95" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="H36" s="29" t="n"/>
+      <c r="I36" s="15" t="n"/>
+    </row>
+    <row r="37" ht="24.95" customHeight="1" s="20">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Thị Ái Phi</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Tiếng Anh </t>
         </is>
       </c>
-      <c r="C36" s="9" t="n"/>
-      <c r="D36" s="13" t="n">
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="13" t="n">
         <v>23</v>
-      </c>
-      <c r="E36" s="13" t="n"/>
-      <c r="F36" s="15" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="G36" s="15" t="n"/>
-      <c r="H36" s="17" t="inlineStr">
-        <is>
-          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D18, 2D19, 2D20, 2D21, 3D19, 3D20, 3D21, 3D22, 3D23</t>
-        </is>
-      </c>
-      <c r="I36" s="15" t="n"/>
-    </row>
-    <row r="37" ht="24.95" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>Lê Thị Hạnh Nhân</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>4D22</t>
-        </is>
-      </c>
-      <c r="D37" s="13" t="n">
-        <v>19</v>
       </c>
       <c r="E37" s="13" t="n"/>
       <c r="F37" s="15" t="inlineStr">
@@ -1533,28 +1617,32 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G37" s="15" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="H37" s="17" t="n"/>
+      <c r="G37" s="15" t="n"/>
+      <c r="H37" s="29" t="inlineStr">
+        <is>
+          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D18, 2D19, 2D20, 2D21, 3D19, 3D20, 3D21, 3D22, 3D23</t>
+        </is>
+      </c>
       <c r="I37" s="15" t="n"/>
     </row>
-    <row r="38" ht="24.95" customHeight="1">
+    <row r="38" ht="24.95" customHeight="1" s="20">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Võ Thị Luyến</t>
+          <t>Lê Thị Hạnh Nhân</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Bộ Môn</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="n"/>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>4D22</t>
+        </is>
+      </c>
       <c r="D38" s="13" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E38" s="13" t="n"/>
       <c r="F38" s="15" t="inlineStr">
@@ -1562,18 +1650,18 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G38" s="15" t="n"/>
-      <c r="H38" s="17" t="inlineStr">
-        <is>
-          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 5D18</t>
-        </is>
-      </c>
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="H38" s="29" t="n"/>
       <c r="I38" s="15" t="n"/>
     </row>
-    <row r="39" ht="24.95" customHeight="1">
+    <row r="39" ht="24.95" customHeight="1" s="20">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Lê Thị Bửu Châu</t>
+          <t>Võ Thị Luyến</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -1592,31 +1680,27 @@
         </is>
       </c>
       <c r="G39" s="15" t="n"/>
-      <c r="H39" s="17" t="inlineStr">
-        <is>
-          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 3D17, 3D18, 3D23</t>
+      <c r="H39" s="29" t="inlineStr">
+        <is>
+          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 5D18</t>
         </is>
       </c>
       <c r="I39" s="15" t="n"/>
     </row>
-    <row r="40" ht="24.95" customHeight="1">
+    <row r="40" ht="24.95" customHeight="1" s="20">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Tý</t>
+          <t>Lê Thị Bửu Châu</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>2D20</t>
-        </is>
-      </c>
+          <t>Bộ Môn</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="n"/>
       <c r="D40" s="13" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E40" s="13" t="n"/>
       <c r="F40" s="15" t="inlineStr">
@@ -1625,23 +1709,31 @@
         </is>
       </c>
       <c r="G40" s="15" t="n"/>
-      <c r="H40" s="17" t="n"/>
+      <c r="H40" s="29" t="inlineStr">
+        <is>
+          <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 3D17, 3D18, 3D23</t>
+        </is>
+      </c>
       <c r="I40" s="15" t="n"/>
     </row>
-    <row r="41" ht="24.95" customHeight="1">
+    <row r="41" ht="24.95" customHeight="1" s="20">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thuận An</t>
+          <t>Nguyễn Thị Tý</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Bộ Môn</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="n"/>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>2D20</t>
+        </is>
+      </c>
       <c r="D41" s="13" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E41" s="13" t="n"/>
       <c r="F41" s="15" t="inlineStr">
@@ -1650,31 +1742,23 @@
         </is>
       </c>
       <c r="G41" s="15" t="n"/>
-      <c r="H41" s="17" t="inlineStr">
-        <is>
-          <t>2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D22, 5D18</t>
-        </is>
-      </c>
+      <c r="H41" s="29" t="n"/>
       <c r="I41" s="15" t="n"/>
     </row>
-    <row r="42" ht="24.95" customHeight="1">
+    <row r="42" ht="24.95" customHeight="1" s="20">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Phạm Hồ Hải Oanh</t>
+          <t>Nguyễn Thuận An</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm</t>
-        </is>
-      </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>3D22</t>
-        </is>
-      </c>
+          <t>Bộ Môn</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="n"/>
       <c r="D42" s="13" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E42" s="13" t="n"/>
       <c r="F42" s="15" t="inlineStr">
@@ -1682,28 +1766,32 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G42" s="15" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="H42" s="17" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="29" t="inlineStr">
+        <is>
+          <t>2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D22, 5D18</t>
+        </is>
+      </c>
       <c r="I42" s="15" t="n"/>
     </row>
-    <row r="43" ht="24.95" customHeight="1">
+    <row r="43" ht="24.95" customHeight="1" s="20">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Lưu Thành Vũ</t>
+          <t>Phạm Hồ Hải Oanh</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Tin học</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="n"/>
+          <t>Chủ Nhiệm</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>3D22</t>
+        </is>
+      </c>
       <c r="D43" s="13" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E43" s="13" t="n"/>
       <c r="F43" s="15" t="inlineStr">
@@ -1711,73 +1799,80 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G43" s="15" t="n"/>
-      <c r="H43" s="17" t="inlineStr">
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n"/>
+      <c r="I43" s="15" t="n"/>
+    </row>
+    <row r="44" ht="24.95" customHeight="1" s="20">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>Lưu Thành Vũ</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>Tin học</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="n"/>
+      <c r="D44" s="24" t="n">
+        <v>23</v>
+      </c>
+      <c r="E44" s="24" t="n"/>
+      <c r="F44" s="25" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G44" s="25" t="n"/>
+      <c r="H44" s="29" t="inlineStr">
         <is>
           <t>3D17, 3D18, 3D19, 3D20, 3D21, 3D22, 3D23, 4D18, 4D19, 4D20, 4D21, 4D22, 5D18, 5D19, 5D20, 5D21, 5D22</t>
         </is>
       </c>
-      <c r="I43" s="15" t="n"/>
-    </row>
-    <row r="44" ht="24.95" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="I44" s="15" t="n"/>
+    </row>
+    <row r="45" ht="24.95" customHeight="1" s="20">
+      <c r="A45" s="26" t="inlineStr">
         <is>
           <t>Lê Hoàng Khoa</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B45" s="27" t="inlineStr">
         <is>
           <t>Thể dục</t>
         </is>
       </c>
-      <c r="C44" s="9" t="n"/>
-      <c r="D44" s="13" t="n">
+      <c r="C45" s="28" t="n"/>
+      <c r="D45" s="28" t="n">
         <v>23</v>
       </c>
-      <c r="E44" s="13" t="n"/>
-      <c r="F44" s="15" t="inlineStr">
+      <c r="E45" s="28" t="n"/>
+      <c r="F45" s="28" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="G44" s="15" t="n"/>
-      <c r="H44" s="17" t="inlineStr">
+      <c r="G45" s="28" t="n"/>
+      <c r="H45" s="29" t="inlineStr">
         <is>
           <t>1D15, 1D16, 1D17, 1D18, 1D19, 1D20, 2D16, 2D17, 2D18, 2D19, 2D20, 2D21, 5D18, 5D19, 5D20, 5D21, 5D22</t>
         </is>
       </c>
-      <c r="I44" s="15" t="n"/>
-    </row>
-    <row r="45" ht="24.95" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>Nguyễn Thị Trúc Ly</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Bộ Môn</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="n"/>
-      <c r="D45" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="E45" s="13" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="F45" s="14" t="n"/>
-      <c r="G45" s="15" t="n"/>
-      <c r="H45" s="17" t="n"/>
-      <c r="I45" s="15" t="inlineStr">
-        <is>
-          <t>Chiều T5, Sáng T6</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="24.95" customHeight="1"/>
+      <c r="I45" s="15" t="n"/>
+    </row>
+    <row r="46" ht="24.95" customHeight="1" s="20">
+      <c r="A46" s="17" t="n"/>
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="19" t="n"/>
+      <c r="D46" s="19" t="n"/>
+      <c r="E46" s="19" t="n"/>
+      <c r="G46" s="19" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1791,15 +1886,15 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="18.75"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.14453125" defaultRowHeight="18"/>
   <cols>
-    <col width="27.5703125" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
-    <col width="9" bestFit="1" customWidth="1" style="1" min="2" max="6"/>
-    <col width="13.5703125" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
-    <col width="9.140625" customWidth="1" style="1" min="8" max="16384"/>
+    <col width="27.57421875" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="9.01171875" bestFit="1" customWidth="1" style="1" min="2" max="6"/>
+    <col width="13.5859375" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
+    <col width="9.14453125" customWidth="1" style="1" min="8" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24.95" customHeight="1">
+    <row r="1" ht="24.95" customHeight="1" s="20">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Môn học</t>
@@ -1831,7 +1926,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="24.95" customHeight="1">
+    <row r="2" ht="24.95" customHeight="1" s="20">
       <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Tiếng Việt</t>
@@ -1853,7 +1948,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="24.95" customHeight="1">
+    <row r="3" ht="24.95" customHeight="1" s="20">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Toán</t>
@@ -1875,7 +1970,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="24.95" customHeight="1">
+    <row r="4" ht="24.95" customHeight="1" s="20">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Hoạt Động Trải Nghiệm</t>
@@ -1897,7 +1992,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" ht="24.95" customHeight="1">
+    <row r="5" ht="24.95" customHeight="1" s="20">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Tiếng Anh</t>
@@ -1919,7 +2014,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="24.95" customHeight="1">
+    <row r="6" ht="24.95" customHeight="1" s="20">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Tự Nhiên và Xã Hội</t>
@@ -1941,7 +2036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="24.95" customHeight="1">
+    <row r="7" ht="24.95" customHeight="1" s="20">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Khoa Học</t>
@@ -1963,7 +2058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="24.95" customHeight="1">
+    <row r="8" ht="24.95" customHeight="1" s="20">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Lịch Sử và Địa Lý</t>
@@ -1985,7 +2080,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="24.95" customHeight="1">
+    <row r="9" ht="24.95" customHeight="1" s="20">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Thể Dục</t>
@@ -2007,7 +2102,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" ht="24.95" customHeight="1">
+    <row r="10" ht="24.95" customHeight="1" s="20">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Âm Nhạc</t>
@@ -2029,7 +2124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" ht="24.95" customHeight="1">
+    <row r="11" ht="24.95" customHeight="1" s="20">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Mỹ Thuật</t>
@@ -2051,7 +2146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" ht="24.95" customHeight="1">
+    <row r="12" ht="24.95" customHeight="1" s="20">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Đạo Đức</t>
@@ -2073,7 +2168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" ht="24.95" customHeight="1">
+    <row r="13" ht="24.95" customHeight="1" s="20">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Tin Học</t>
@@ -2095,7 +2190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" ht="24.95" customHeight="1">
+    <row r="14" ht="24.95" customHeight="1" s="20">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Công Nghệ</t>
@@ -2117,7 +2212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" ht="24.95" customHeight="1">
+    <row r="15" ht="24.95" customHeight="1" s="20">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Toán Tăng Cường</t>
@@ -2139,7 +2234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="24.95" customHeight="1">
+    <row r="16" ht="24.95" customHeight="1" s="20">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Tiếng Việt Tăng Cường</t>
@@ -2161,7 +2256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="24.95" customHeight="1">
+    <row r="17" ht="24.95" customHeight="1" s="20">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Kỹ Năng Sống</t>

</xml_diff>

<commit_message>
School file: abbreviations and short names as on the school's board
Fill the column Tên trong TKB of CHƯƠNG TRÌNH HỌC (T, AN, GDTC, Tin,
LS&ĐL, keeping the existing HĐTN, TNXH, TV tăng cường) and the column
Tên Viết Tắt of NHÂN SỰ for all 44 people, taken from the school's
hand-made board timetable, so TKB_toan_truong.xlsx reads like it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SYSHWKNfUbV9f2WQ9CocTD
</commit_message>
<xml_diff>
--- a/data/INPUT_V8.xlsx
+++ b/data/INPUT_V8.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NHÂN SỰ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CHƯƠNG TRÌNH HỌC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NHÂN SỰ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHƯƠNG TRÌNH HỌC" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="33.62890625" bestFit="1" customWidth="1" style="20" min="1" max="1"/>
@@ -640,6 +640,7 @@
     <col width="10.35546875" bestFit="1" customWidth="1" style="19" min="7" max="7"/>
     <col width="40" customWidth="1" style="20" min="8" max="8"/>
     <col width="22" customWidth="1" style="20" min="9" max="9"/>
+    <col width="14" customWidth="1" style="20" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24.95" customHeight="1" s="20">
@@ -688,6 +689,11 @@
           <t>Buổi Nghỉ</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Tên Viết Tắt</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="24.95" customHeight="1" s="20">
       <c r="A2" s="6" t="inlineStr">
@@ -713,6 +719,11 @@
         </is>
       </c>
       <c r="I2" s="15" t="n"/>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>Tâm</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="24.95" customHeight="1" s="20">
       <c r="A3" s="6" t="inlineStr">
@@ -738,6 +749,11 @@
       <c r="G3" s="15" t="n"/>
       <c r="H3" s="29" t="n"/>
       <c r="I3" s="15" t="n"/>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>T.Ngọc</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="24.95" customHeight="1" s="20">
       <c r="A4" s="6" t="inlineStr">
@@ -763,6 +779,11 @@
       <c r="G4" s="15" t="n"/>
       <c r="H4" s="29" t="n"/>
       <c r="I4" s="15" t="n"/>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Dương</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="24.95" customHeight="1" s="20">
       <c r="A5" s="6" t="inlineStr">
@@ -788,6 +809,11 @@
         </is>
       </c>
       <c r="I5" s="15" t="n"/>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>T.Anh</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="24.95" customHeight="1" s="20">
       <c r="A6" s="6" t="inlineStr">
@@ -813,6 +839,11 @@
       <c r="G6" s="15" t="n"/>
       <c r="H6" s="29" t="n"/>
       <c r="I6" s="15" t="n"/>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>Viễn</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24.95" customHeight="1" s="20">
       <c r="A7" s="6" t="inlineStr">
@@ -838,6 +869,11 @@
       <c r="G7" s="15" t="n"/>
       <c r="H7" s="29" t="n"/>
       <c r="I7" s="15" t="n"/>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>Lộc</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="24.95" customHeight="1" s="20">
       <c r="A8" s="6" t="inlineStr">
@@ -863,6 +899,11 @@
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="29" t="n"/>
       <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>Lạc</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="24.95" customHeight="1" s="20">
       <c r="A9" s="6" t="inlineStr">
@@ -888,6 +929,11 @@
       <c r="G9" s="15" t="n"/>
       <c r="H9" s="29" t="n"/>
       <c r="I9" s="15" t="n"/>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>Phụng</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="24.95" customHeight="1" s="20">
       <c r="A10" s="6" t="inlineStr">
@@ -913,6 +959,11 @@
         </is>
       </c>
       <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>Hoà</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="24.95" customHeight="1" s="20">
       <c r="A11" s="6" t="inlineStr">
@@ -938,6 +989,11 @@
       <c r="G11" s="15" t="n"/>
       <c r="H11" s="29" t="n"/>
       <c r="I11" s="15" t="n"/>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>Dung</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="24.95" customHeight="1" s="20">
       <c r="A12" s="6" t="inlineStr">
@@ -967,6 +1023,11 @@
       </c>
       <c r="H12" s="29" t="n"/>
       <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="inlineStr">
+        <is>
+          <t>Vân</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="24.95" customHeight="1" s="20">
       <c r="A13" s="6" t="inlineStr">
@@ -992,6 +1053,11 @@
         </is>
       </c>
       <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>Sa</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="24.95" customHeight="1" s="20">
       <c r="A14" s="6" t="inlineStr">
@@ -1017,6 +1083,11 @@
       <c r="G14" s="15" t="n"/>
       <c r="H14" s="29" t="n"/>
       <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="inlineStr">
+        <is>
+          <t>H.Vi</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="24.95" customHeight="1" s="20">
       <c r="A15" s="6" t="inlineStr">
@@ -1042,6 +1113,11 @@
       <c r="G15" s="15" t="n"/>
       <c r="H15" s="29" t="n"/>
       <c r="I15" s="15" t="n"/>
+      <c r="J15" s="15" t="inlineStr">
+        <is>
+          <t>Oanh</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="24.95" customHeight="1" s="20">
       <c r="A16" s="6" t="inlineStr">
@@ -1067,6 +1143,11 @@
         </is>
       </c>
       <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="inlineStr">
+        <is>
+          <t>Thịnh</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="24.95" customHeight="1" s="20">
       <c r="A17" s="6" t="inlineStr">
@@ -1096,6 +1177,11 @@
       </c>
       <c r="H17" s="29" t="n"/>
       <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="inlineStr">
+        <is>
+          <t>K.Ngọc</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="24.95" customHeight="1" s="20">
       <c r="A18" s="6" t="inlineStr">
@@ -1121,6 +1207,11 @@
       <c r="G18" s="15" t="n"/>
       <c r="H18" s="29" t="n"/>
       <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="inlineStr">
+        <is>
+          <t>T.Trang</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="24.95" customHeight="1" s="20">
       <c r="A19" s="6" t="inlineStr">
@@ -1146,6 +1237,11 @@
       <c r="G19" s="15" t="n"/>
       <c r="H19" s="29" t="n"/>
       <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="inlineStr">
+        <is>
+          <t>Nhung</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="24.95" customHeight="1" s="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1171,6 +1267,11 @@
       <c r="G20" s="15" t="n"/>
       <c r="H20" s="29" t="n"/>
       <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="inlineStr">
+        <is>
+          <t>Thảo</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="24.95" customHeight="1" s="20">
       <c r="A21" s="6" t="inlineStr">
@@ -1196,6 +1297,11 @@
       <c r="G21" s="15" t="n"/>
       <c r="H21" s="29" t="n"/>
       <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="inlineStr">
+        <is>
+          <t>Trân</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="24.95" customHeight="1" s="20">
       <c r="A22" s="6" t="inlineStr">
@@ -1221,6 +1327,11 @@
       <c r="G22" s="15" t="n"/>
       <c r="H22" s="29" t="n"/>
       <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="inlineStr">
+        <is>
+          <t>Tri</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="24.95" customHeight="1" s="20">
       <c r="A23" s="6" t="inlineStr">
@@ -1246,6 +1357,11 @@
       <c r="G23" s="15" t="n"/>
       <c r="H23" s="29" t="n"/>
       <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="inlineStr">
+        <is>
+          <t>Nuôi</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="24.95" customHeight="1" s="20">
       <c r="A24" s="6" t="inlineStr">
@@ -1281,6 +1397,11 @@
       <c r="I24" s="15" t="inlineStr">
         <is>
           <t>2 buổi chiều</t>
+        </is>
+      </c>
+      <c r="J24" s="15" t="inlineStr">
+        <is>
+          <t>Mai</t>
         </is>
       </c>
     </row>
@@ -1308,6 +1429,11 @@
         </is>
       </c>
       <c r="I25" s="15" t="n"/>
+      <c r="J25" s="15" t="inlineStr">
+        <is>
+          <t>Vi</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="24.95" customHeight="1" s="20">
       <c r="A26" s="6" t="inlineStr">
@@ -1333,6 +1459,11 @@
       <c r="G26" s="15" t="n"/>
       <c r="H26" s="29" t="n"/>
       <c r="I26" s="15" t="n"/>
+      <c r="J26" s="15" t="inlineStr">
+        <is>
+          <t>B.Huyền</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="24.95" customHeight="1" s="20">
       <c r="A27" s="6" t="inlineStr">
@@ -1358,6 +1489,11 @@
       <c r="G27" s="15" t="n"/>
       <c r="H27" s="29" t="n"/>
       <c r="I27" s="15" t="n"/>
+      <c r="J27" s="15" t="inlineStr">
+        <is>
+          <t>A.Thư</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="24.95" customHeight="1" s="20">
       <c r="A28" s="6" t="inlineStr">
@@ -1383,6 +1519,11 @@
       <c r="G28" s="15" t="n"/>
       <c r="H28" s="29" t="n"/>
       <c r="I28" s="15" t="n"/>
+      <c r="J28" s="15" t="inlineStr">
+        <is>
+          <t>T.Huyền</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="24.95" customHeight="1" s="20">
       <c r="A29" s="6" t="inlineStr">
@@ -1408,6 +1549,11 @@
         </is>
       </c>
       <c r="I29" s="15" t="n"/>
+      <c r="J29" s="15" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="24.95" customHeight="1" s="20">
       <c r="A30" s="6" t="inlineStr">
@@ -1433,6 +1579,11 @@
       <c r="G30" s="15" t="n"/>
       <c r="H30" s="29" t="n"/>
       <c r="I30" s="15" t="n"/>
+      <c r="J30" s="15" t="inlineStr">
+        <is>
+          <t>Dân</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="24.95" customHeight="1" s="20">
       <c r="A31" s="6" t="inlineStr">
@@ -1458,6 +1609,11 @@
       <c r="G31" s="15" t="n"/>
       <c r="H31" s="29" t="n"/>
       <c r="I31" s="15" t="n"/>
+      <c r="J31" s="15" t="inlineStr">
+        <is>
+          <t>Võ Ly</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="24.95" customHeight="1" s="20">
       <c r="A32" s="6" t="inlineStr">
@@ -1483,6 +1639,11 @@
       <c r="G32" s="15" t="n"/>
       <c r="H32" s="29" t="n"/>
       <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="inlineStr">
+        <is>
+          <t>Hoàng Vy</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="24.95" customHeight="1" s="20">
       <c r="A33" s="6" t="inlineStr">
@@ -1508,6 +1669,11 @@
       <c r="G33" s="15" t="n"/>
       <c r="H33" s="29" t="n"/>
       <c r="I33" s="15" t="n"/>
+      <c r="J33" s="15" t="inlineStr">
+        <is>
+          <t>Thủy</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="24.95" customHeight="1" s="20">
       <c r="A34" s="6" t="inlineStr">
@@ -1539,6 +1705,11 @@
       <c r="I34" s="15" t="inlineStr">
         <is>
           <t>Chiều T5, Sáng T6</t>
+        </is>
+      </c>
+      <c r="J34" s="15" t="inlineStr">
+        <is>
+          <t>N.Ly</t>
         </is>
       </c>
     </row>
@@ -1566,6 +1737,11 @@
         </is>
       </c>
       <c r="I35" s="15" t="n"/>
+      <c r="J35" s="15" t="inlineStr">
+        <is>
+          <t>Quỳnh</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="24.95" customHeight="1" s="20">
       <c r="A36" s="6" t="inlineStr">
@@ -1595,6 +1771,11 @@
       </c>
       <c r="H36" s="29" t="n"/>
       <c r="I36" s="15" t="n"/>
+      <c r="J36" s="15" t="inlineStr">
+        <is>
+          <t>Hạnh</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="24.95" customHeight="1" s="20">
       <c r="A37" s="6" t="inlineStr">
@@ -1624,6 +1805,11 @@
         </is>
       </c>
       <c r="I37" s="15" t="n"/>
+      <c r="J37" s="15" t="inlineStr">
+        <is>
+          <t>Phi</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="24.95" customHeight="1" s="20">
       <c r="A38" s="6" t="inlineStr">
@@ -1657,6 +1843,11 @@
       </c>
       <c r="H38" s="29" t="n"/>
       <c r="I38" s="15" t="n"/>
+      <c r="J38" s="15" t="inlineStr">
+        <is>
+          <t>Nhân</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="24.95" customHeight="1" s="20">
       <c r="A39" s="6" t="inlineStr">
@@ -1686,6 +1877,11 @@
         </is>
       </c>
       <c r="I39" s="15" t="n"/>
+      <c r="J39" s="15" t="inlineStr">
+        <is>
+          <t>Luyến</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="24.95" customHeight="1" s="20">
       <c r="A40" s="6" t="inlineStr">
@@ -1715,6 +1911,11 @@
         </is>
       </c>
       <c r="I40" s="15" t="n"/>
+      <c r="J40" s="15" t="inlineStr">
+        <is>
+          <t>Châu</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="24.95" customHeight="1" s="20">
       <c r="A41" s="6" t="inlineStr">
@@ -1744,6 +1945,11 @@
       <c r="G41" s="15" t="n"/>
       <c r="H41" s="29" t="n"/>
       <c r="I41" s="15" t="n"/>
+      <c r="J41" s="15" t="inlineStr">
+        <is>
+          <t>Tý</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="24.95" customHeight="1" s="20">
       <c r="A42" s="6" t="inlineStr">
@@ -1773,6 +1979,11 @@
         </is>
       </c>
       <c r="I42" s="15" t="n"/>
+      <c r="J42" s="15" t="inlineStr">
+        <is>
+          <t>An</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="24.95" customHeight="1" s="20">
       <c r="A43" s="6" t="inlineStr">
@@ -1806,6 +2017,11 @@
       </c>
       <c r="H43" s="29" t="n"/>
       <c r="I43" s="15" t="n"/>
+      <c r="J43" s="15" t="inlineStr">
+        <is>
+          <t>Oanh</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="24.95" customHeight="1" s="20">
       <c r="A44" s="21" t="inlineStr">
@@ -1835,6 +2051,11 @@
         </is>
       </c>
       <c r="I44" s="15" t="n"/>
+      <c r="J44" s="15" t="inlineStr">
+        <is>
+          <t>Vũ</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="24.95" customHeight="1" s="20">
       <c r="A45" s="26" t="inlineStr">
@@ -1864,6 +2085,11 @@
         </is>
       </c>
       <c r="I45" s="15" t="n"/>
+      <c r="J45" s="15" t="inlineStr">
+        <is>
+          <t>Khoa</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="24.95" customHeight="1" s="20">
       <c r="A46" s="17" t="n"/>
@@ -1885,12 +2111,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.14453125" defaultRowHeight="18"/>
   <cols>
     <col width="27.57421875" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="9.01171875" bestFit="1" customWidth="1" style="1" min="2" max="6"/>
-    <col width="13.5859375" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
+    <col width="16" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
     <col width="9.14453125" customWidth="1" style="1" min="8" max="16384"/>
   </cols>
   <sheetData>
@@ -1925,6 +2151,11 @@
           <t>Khối 5</t>
         </is>
       </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Tên trong TKB</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="24.95" customHeight="1" s="20">
       <c r="A2" s="4" t="inlineStr">
@@ -1947,6 +2178,7 @@
       <c r="F2" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="G2" s="4" t="n"/>
     </row>
     <row r="3" ht="24.95" customHeight="1" s="20">
       <c r="A3" s="2" t="inlineStr">
@@ -1969,6 +2201,11 @@
       <c r="F3" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="24.95" customHeight="1" s="20">
       <c r="A4" s="4" t="inlineStr">
@@ -1991,6 +2228,11 @@
       <c r="F4" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>HĐTN</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="24.95" customHeight="1" s="20">
       <c r="A5" s="2" t="inlineStr">
@@ -2013,6 +2255,7 @@
       <c r="F5" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6" ht="24.95" customHeight="1" s="20">
       <c r="A6" s="4" t="inlineStr">
@@ -2035,6 +2278,11 @@
       <c r="F6" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>TNXH</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24.95" customHeight="1" s="20">
       <c r="A7" s="2" t="inlineStr">
@@ -2057,6 +2305,7 @@
       <c r="F7" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8" ht="24.95" customHeight="1" s="20">
       <c r="A8" s="4" t="inlineStr">
@@ -2079,6 +2328,11 @@
       <c r="F8" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>LS&amp;ĐL</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="24.95" customHeight="1" s="20">
       <c r="A9" s="2" t="inlineStr">
@@ -2101,6 +2355,11 @@
       <c r="F9" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>GDTC</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="24.95" customHeight="1" s="20">
       <c r="A10" s="4" t="inlineStr">
@@ -2123,6 +2382,11 @@
       <c r="F10" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="24.95" customHeight="1" s="20">
       <c r="A11" s="2" t="inlineStr">
@@ -2145,6 +2409,7 @@
       <c r="F11" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12" ht="24.95" customHeight="1" s="20">
       <c r="A12" s="4" t="inlineStr">
@@ -2167,6 +2432,7 @@
       <c r="F12" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="G12" s="4" t="n"/>
     </row>
     <row r="13" ht="24.95" customHeight="1" s="20">
       <c r="A13" s="2" t="inlineStr">
@@ -2189,6 +2455,11 @@
       <c r="F13" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Tin</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="24.95" customHeight="1" s="20">
       <c r="A14" s="4" t="inlineStr">
@@ -2211,6 +2482,7 @@
       <c r="F14" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="G14" s="4" t="n"/>
     </row>
     <row r="15" ht="24.95" customHeight="1" s="20">
       <c r="A15" s="2" t="inlineStr">
@@ -2233,6 +2505,7 @@
       <c r="F15" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16" ht="24.95" customHeight="1" s="20">
       <c r="A16" s="4" t="inlineStr">
@@ -2255,6 +2528,11 @@
       <c r="F16" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>TV tăng cường</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="24.95" customHeight="1" s="20">
       <c r="A17" s="2" t="inlineStr">
@@ -2277,6 +2555,7 @@
       <c r="F17" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G17" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>